<commit_message>
added list for some columns
</commit_message>
<xml_diff>
--- a/importing excel and changing/Outputs/check_this.xlsx
+++ b/importing excel and changing/Outputs/check_this.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S60"/>
+  <dimension ref="A1:T60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -510,6 +510,11 @@
       <c r="S1" t="inlineStr">
         <is>
           <t>col-8</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>DictionaryValues</t>
         </is>
       </c>
     </row>
@@ -561,6 +566,11 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -614,6 +624,11 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -675,6 +690,11 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>['Male', 'Female', nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -728,6 +748,11 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -797,6 +822,11 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>['Hispanic or Latino', 'Not Hispanic or Latino', 'Not Reported', 'Unknown', nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -846,6 +876,11 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -895,6 +930,11 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -944,6 +984,11 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -993,6 +1038,11 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1042,6 +1092,11 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1091,6 +1146,11 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1140,6 +1200,11 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1189,6 +1254,11 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1238,6 +1308,11 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1287,6 +1362,11 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1336,6 +1416,11 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1389,6 +1474,11 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1458,6 +1548,11 @@
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>['Adverse Event', 'Site Error', 'Not Clinically Indicated', 'Other, Specify', nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1507,6 +1602,11 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1572,6 +1672,11 @@
       </c>
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>[0, 1, 2, 3, 4, 5, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1621,6 +1726,11 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1674,6 +1784,11 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1723,6 +1838,11 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1776,6 +1896,11 @@
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1829,6 +1954,11 @@
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1882,6 +2012,11 @@
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1935,6 +2070,11 @@
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1988,6 +2128,11 @@
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2037,6 +2182,11 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2086,6 +2236,11 @@
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2135,6 +2290,11 @@
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2184,6 +2344,11 @@
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2233,6 +2398,11 @@
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2286,6 +2456,11 @@
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2335,6 +2510,11 @@
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2384,6 +2564,11 @@
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2433,6 +2618,11 @@
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2482,6 +2672,11 @@
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2555,6 +2750,11 @@
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr"/>
       <c r="S40" t="inlineStr"/>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>['Grade 1', 'Grade 2', 'Grade 3', 'Grade 4', 'Grade 5', nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2628,6 +2828,11 @@
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr"/>
       <c r="S41" t="inlineStr"/>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>['Unrelated', 'Unlikely Related', 'Possibly Related', 'Probably Related', 'Definitely Related', nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2711,6 +2916,11 @@
       <c r="S42" t="inlineStr">
         <is>
           <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>['Dose Not Changed', 'Drug Withdrawn', 'Drug Delayed/Interrupted', 'Dose Reduced', 'Dose Increased', 'Dose Rate Reduced', 'Unknown', 'Not Applicable']</t>
         </is>
       </c>
     </row>
@@ -2786,6 +2996,11 @@
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr"/>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>['Unrelated', 'Unlikely Related', 'Possibly Related', 'Probably Related', 'Definitely Related', nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2871,6 +3086,11 @@
           <t>Not Applicable</t>
         </is>
       </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>['Dose Not Changed', 'Drug Withdrawn', 'Drug Delayed/Interrupted', 'Dose Reduced', 'Dose Increased', 'Dose Rate Reduced', 'Unknown', 'Not Applicable']</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2948,6 +3168,11 @@
       </c>
       <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr"/>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>['Recovered/Resolved', 'Recovered/Resolved with Sequelae', 'Recovering/Resolving', 'Not Recovered/Not Resolved', 'Fatal', 'Unknown', nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2997,6 +3222,11 @@
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr"/>
       <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3042,6 +3272,11 @@
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3091,6 +3326,11 @@
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr"/>
       <c r="S48" t="inlineStr"/>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3140,6 +3380,11 @@
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr"/>
       <c r="S49" t="inlineStr"/>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3189,6 +3434,11 @@
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr"/>
       <c r="S50" t="inlineStr"/>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3242,6 +3492,11 @@
       <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr"/>
       <c r="S51" t="inlineStr"/>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3291,6 +3546,11 @@
       <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr"/>
       <c r="S52" t="inlineStr"/>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3340,6 +3600,11 @@
       <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr"/>
       <c r="S53" t="inlineStr"/>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3389,6 +3654,11 @@
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr"/>
       <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3438,6 +3708,11 @@
       <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr"/>
       <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3487,6 +3762,11 @@
       <c r="Q56" t="inlineStr"/>
       <c r="R56" t="inlineStr"/>
       <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3536,6 +3816,11 @@
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr"/>
       <c r="S57" t="inlineStr"/>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3585,6 +3870,11 @@
       <c r="Q58" t="inlineStr"/>
       <c r="R58" t="inlineStr"/>
       <c r="S58" t="inlineStr"/>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3634,6 +3924,11 @@
       <c r="Q59" t="inlineStr"/>
       <c r="R59" t="inlineStr"/>
       <c r="S59" t="inlineStr"/>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3683,6 +3978,11 @@
       <c r="Q60" t="inlineStr"/>
       <c r="R60" t="inlineStr"/>
       <c r="S60" t="inlineStr"/>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>[nan, nan, nan, nan, nan, nan, nan, nan]</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>